<commit_message>
feat: add CAM report template file for standardized assessment exports
</commit_message>
<xml_diff>
--- a/attached_assets/CAM_format/CAM_REPORT_FORMAT.xlsx
+++ b/attached_assets/CAM_format/CAM_REPORT_FORMAT.xlsx
@@ -358,7 +358,7 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -702,6 +702,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1297,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="45.6640625" customWidth="1" min="1" max="1"/>
@@ -1731,6 +1737,7 @@
       <c r="B15" s="70" t="n">
         <v>34259</v>
       </c>
+      <c r="C15" s="95" t="n"/>
       <c r="D15" s="1" t="n"/>
       <c r="E15" s="25" t="inlineStr">
         <is>
@@ -1757,6 +1764,7 @@
         <f>YEAR(TODAY())-YEAR(B15)-IF(DATE(YEAR(TODAY()),MONTH(B15),DAY(B15))&gt;TODAY(),1,0)&amp;" YEARS OLD"</f>
         <v/>
       </c>
+      <c r="C16" s="95" t="n"/>
       <c r="D16" s="1" t="n"/>
       <c r="E16" s="25" t="inlineStr">
         <is>
@@ -1803,6 +1811,7 @@
         </is>
       </c>
       <c r="B18" s="73" t="n"/>
+      <c r="C18" s="95" t="n"/>
       <c r="D18" s="1" t="n"/>
       <c r="E18" s="22" t="n"/>
       <c r="F18" s="22" t="n"/>
@@ -1818,7 +1827,7 @@
           <t>HOUSE TYPE: (OWNED/RENTED/HOSTEL)</t>
         </is>
       </c>
-      <c r="B19" s="74" t="n"/>
+      <c r="B19" s="76" t="n"/>
       <c r="C19" s="95" t="n"/>
       <c r="D19" s="1" t="n"/>
       <c r="E19" s="72" t="inlineStr">
@@ -1839,11 +1848,12 @@
           <t>CURRENT ADDRESS</t>
         </is>
       </c>
-      <c r="B20" s="74" t="inlineStr">
+      <c r="B20" s="76" t="inlineStr">
         <is>
           <t>current address</t>
         </is>
       </c>
+      <c r="C20" s="95" t="n"/>
       <c r="D20" s="1" t="n"/>
       <c r="E20" s="72" t="n"/>
       <c r="F20" s="28" t="n">
@@ -1903,6 +1913,7 @@
         </is>
       </c>
       <c r="B22" s="74" t="n"/>
+      <c r="C22" s="95" t="n"/>
       <c r="D22" s="1" t="n"/>
       <c r="E22" s="72" t="inlineStr">
         <is>
@@ -1932,7 +1943,7 @@
           <t>WORKING ADDRESS</t>
         </is>
       </c>
-      <c r="B23" s="67" t="inlineStr">
+      <c r="B23" s="68" t="inlineStr">
         <is>
           <t>working address</t>
         </is>
@@ -1967,11 +1978,12 @@
           <t>PERMANENT ADDRESS</t>
         </is>
       </c>
-      <c r="B24" s="74" t="inlineStr">
+      <c r="B24" s="76" t="inlineStr">
         <is>
           <t>permanent address</t>
         </is>
       </c>
+      <c r="C24" s="95" t="n"/>
       <c r="D24" s="1" t="n"/>
       <c r="E24" s="72" t="inlineStr">
         <is>
@@ -2001,6 +2013,8 @@
           <t>PROFESSION DETAILS</t>
         </is>
       </c>
+      <c r="B25" s="94" t="n"/>
+      <c r="C25" s="95" t="n"/>
       <c r="D25" s="1" t="n"/>
       <c r="E25" s="72" t="inlineStr">
         <is>
@@ -2030,7 +2044,7 @@
           <t>DOCTOR / CA / CS</t>
         </is>
       </c>
-      <c r="B26" s="94" t="n"/>
+      <c r="B26" s="118" t="n"/>
       <c r="C26" s="95" t="n"/>
       <c r="D26" s="1" t="n"/>
       <c r="E26" s="72" t="inlineStr">
@@ -2066,6 +2080,7 @@
           <t>MBBS | MS</t>
         </is>
       </c>
+      <c r="C27" s="95" t="n"/>
       <c r="D27" s="1" t="n"/>
       <c r="E27" s="72" t="n"/>
       <c r="F27" s="106">
@@ -2132,6 +2147,7 @@
           <t>7 YEARS</t>
         </is>
       </c>
+      <c r="C29" s="95" t="n"/>
       <c r="D29" s="1" t="n"/>
       <c r="E29" s="35" t="n"/>
       <c r="F29" s="108" t="n"/>
@@ -2173,6 +2189,7 @@
         </is>
       </c>
       <c r="B31" s="68" t="n"/>
+      <c r="C31" s="95" t="n"/>
       <c r="D31" s="1" t="n"/>
       <c r="E31" s="72" t="inlineStr">
         <is>
@@ -2192,6 +2209,8 @@
           <t>BANKING DETAILS</t>
         </is>
       </c>
+      <c r="B32" s="94" t="n"/>
+      <c r="C32" s="95" t="n"/>
       <c r="D32" s="1" t="n"/>
       <c r="E32" s="75" t="inlineStr">
         <is>
@@ -2229,7 +2248,8 @@
           <t>CIBIL SCORE</t>
         </is>
       </c>
-      <c r="B33" s="94" t="n"/>
+      <c r="B33" s="119" t="n"/>
+      <c r="C33" s="94" t="n"/>
       <c r="D33" s="1" t="n"/>
       <c r="E33" s="75" t="inlineStr">
         <is>
@@ -2297,6 +2317,7 @@
         <f>COUNTA(F3:F10)&amp;" | LOANS"</f>
         <v/>
       </c>
+      <c r="C36" s="95" t="n"/>
       <c r="D36" s="1" t="n"/>
       <c r="E36" s="42" t="inlineStr">
         <is>
@@ -2421,6 +2442,7 @@
         </is>
       </c>
       <c r="B41" s="81" t="n"/>
+      <c r="C41" s="95" t="n"/>
       <c r="D41" s="1" t="n"/>
       <c r="E41" s="45" t="inlineStr">
         <is>
@@ -2457,6 +2479,8 @@
           <t>NOMINEE DETAILS</t>
         </is>
       </c>
+      <c r="B43" s="94" t="n"/>
+      <c r="C43" s="95" t="n"/>
       <c r="D43" s="1" t="n"/>
       <c r="E43" s="89" t="inlineStr">
         <is>
@@ -2518,6 +2542,7 @@
         </is>
       </c>
       <c r="B46" s="68" t="n"/>
+      <c r="C46" s="95" t="n"/>
       <c r="D46" s="1" t="n"/>
       <c r="E46" s="49" t="n"/>
       <c r="F46" s="50" t="n"/>
@@ -2533,6 +2558,8 @@
           <t>REFERANCE</t>
         </is>
       </c>
+      <c r="B47" s="94" t="n"/>
+      <c r="C47" s="95" t="n"/>
       <c r="D47" s="1" t="n"/>
       <c r="E47" s="49" t="n"/>
       <c r="F47" s="50" t="n"/>
@@ -2598,6 +2625,7 @@
         </is>
       </c>
       <c r="B51" s="68" t="n"/>
+      <c r="C51" s="95" t="n"/>
       <c r="D51" s="1" t="n"/>
       <c r="E51" s="53" t="n"/>
       <c r="F51" s="54" t="n"/>
@@ -2685,6 +2713,7 @@
         </is>
       </c>
       <c r="B56" s="82" t="n"/>
+      <c r="C56" s="95" t="n"/>
       <c r="D56" s="1" t="n"/>
       <c r="E56" s="114" t="n"/>
       <c r="F56" s="116" t="n"/>
@@ -2735,6 +2764,7 @@
         </is>
       </c>
       <c r="B59" s="82" t="n"/>
+      <c r="C59" s="95" t="n"/>
       <c r="D59" s="1" t="n"/>
       <c r="E59" s="117" t="n"/>
       <c r="F59" s="113" t="n"/>
@@ -2768,6 +2798,7 @@
         </is>
       </c>
       <c r="B61" s="82" t="n"/>
+      <c r="C61" s="95" t="n"/>
       <c r="D61" s="1" t="n"/>
     </row>
     <row r="62" ht="178.05" customHeight="1">
@@ -2779,14 +2810,7 @@
       <c r="B62" s="82" t="n"/>
       <c r="C62" s="95" t="n"/>
     </row>
-    <row r="63" ht="217.95" customHeight="1">
-      <c r="A63" s="62" t="inlineStr">
-        <is>
-          <t>CREDIT REMARK</t>
-        </is>
-      </c>
-      <c r="B63" s="92" t="n"/>
-    </row>
+    <row r="63" ht="217.95" customHeight="1"/>
     <row r="64"/>
     <row r="65"/>
     <row r="66"/>
@@ -2823,16 +2847,15 @@
     <row r="97"/>
     <row r="98"/>
     <row r="99"/>
-    <row r="101"/>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="54">
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="A25:C25"/>
-    <mergeCell ref="F33:K33"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B62:C62"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="B7:C7"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B7:C7"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B46:C46"/>
     <mergeCell ref="B22:C22"/>
@@ -2840,14 +2863,17 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B56:C56"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="F28:K28"/>
     <mergeCell ref="A32:C32"/>
+    <mergeCell ref="B42:C42"/>
     <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="A43:C43"/>
@@ -2855,20 +2881,27 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="E19:K19"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B15:C15"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="E30:K30"/>
-    <mergeCell ref="B20:C20"/>
     <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="E35:G35"/>
     <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <dataValidations count="4">

</xml_diff>